<commit_message>
2026-07-19 Changes to Predictions dashboard, including carousel
</commit_message>
<xml_diff>
--- a/Python/Activities/data.xlsx
+++ b/Python/Activities/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Activities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3954E254-AF62-4E91-AA5F-432F94DF022A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24DCA9D0-19F1-4D56-9B93-8B080CCDC297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{707279AB-A7E9-4A68-BEA1-90F4DD1BCF34}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="74">
   <si>
     <t>walk</t>
   </si>
@@ -237,19 +237,19 @@
     <t>other</t>
   </si>
   <si>
-    <t>Sum</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Running Total</t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
     <t>11'21"</t>
+  </si>
+  <si>
+    <t>11'49"</t>
+  </si>
+  <si>
+    <t>10'58"</t>
+  </si>
+  <si>
+    <t>10'04"</t>
+  </si>
+  <si>
+    <t>11'26"</t>
   </si>
 </sst>
 </file>
@@ -257,7 +257,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="hh:mm;@"/>
+    <numFmt numFmtId="164" formatCode="hh:mm;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -293,7 +293,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -609,7 +609,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F196B904-6553-42BC-A222-B01279AC4ED1}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Q95"/>
+  <dimension ref="A1:Q108"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -4011,7 +4011,7 @@
         <v>7278</v>
       </c>
       <c r="J91" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="K91" s="2">
         <v>124</v>
@@ -4100,6 +4100,371 @@
         <v>60</v>
       </c>
       <c r="E95" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>46208</v>
+      </c>
+      <c r="B96" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C96" t="s">
+        <v>2</v>
+      </c>
+      <c r="D96" s="2">
+        <v>60</v>
+      </c>
+      <c r="E96" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>46208</v>
+      </c>
+      <c r="B97" s="4">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="C97" t="s">
+        <v>1</v>
+      </c>
+      <c r="D97" s="2">
+        <v>60</v>
+      </c>
+      <c r="E97" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>46212</v>
+      </c>
+      <c r="B98" s="4">
+        <v>0.49722222222222223</v>
+      </c>
+      <c r="C98" t="s">
+        <v>0</v>
+      </c>
+      <c r="D98" s="2">
+        <v>3844</v>
+      </c>
+      <c r="E98" t="s">
+        <v>22</v>
+      </c>
+      <c r="F98" s="2">
+        <v>30</v>
+      </c>
+      <c r="G98" s="2">
+        <v>662</v>
+      </c>
+      <c r="H98" s="3">
+        <v>5.42</v>
+      </c>
+      <c r="I98" s="2">
+        <v>7393</v>
+      </c>
+      <c r="J98" t="s">
+        <v>70</v>
+      </c>
+      <c r="K98" s="2">
+        <v>128</v>
+      </c>
+      <c r="L98" s="2">
+        <v>0</v>
+      </c>
+      <c r="M98" s="2">
+        <v>34</v>
+      </c>
+      <c r="N98" s="2">
+        <v>6</v>
+      </c>
+      <c r="O98" s="2">
+        <v>21</v>
+      </c>
+      <c r="P98" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q98" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>46217</v>
+      </c>
+      <c r="B99" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C99" t="s">
+        <v>2</v>
+      </c>
+      <c r="D99" s="2">
+        <v>60</v>
+      </c>
+      <c r="E99" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B100" s="4">
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="C100" t="s">
+        <v>1</v>
+      </c>
+      <c r="D100" s="2">
+        <v>60</v>
+      </c>
+      <c r="E100" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B101" s="4">
+        <v>0.43055555555555558</v>
+      </c>
+      <c r="C101" t="s">
+        <v>0</v>
+      </c>
+      <c r="D101" s="2">
+        <v>3737</v>
+      </c>
+      <c r="E101" t="s">
+        <v>22</v>
+      </c>
+      <c r="F101" s="2">
+        <v>71</v>
+      </c>
+      <c r="G101" s="2">
+        <v>760</v>
+      </c>
+      <c r="H101" s="3">
+        <v>5.68</v>
+      </c>
+      <c r="I101" s="2">
+        <v>7306</v>
+      </c>
+      <c r="J101" t="s">
+        <v>71</v>
+      </c>
+      <c r="K101" s="2">
+        <v>135</v>
+      </c>
+      <c r="L101" s="2">
+        <v>0</v>
+      </c>
+      <c r="M101" s="2">
+        <v>69</v>
+      </c>
+      <c r="N101" s="2">
+        <v>6</v>
+      </c>
+      <c r="O101" s="2">
+        <v>18</v>
+      </c>
+      <c r="P101" s="2">
+        <v>24</v>
+      </c>
+      <c r="Q101" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>46218</v>
+      </c>
+      <c r="B102" s="4">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C102" t="s">
+        <v>2</v>
+      </c>
+      <c r="D102" s="2">
+        <v>60</v>
+      </c>
+      <c r="E102" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>46219</v>
+      </c>
+      <c r="B103" s="4">
+        <v>0.4375</v>
+      </c>
+      <c r="C103" t="s">
+        <v>2</v>
+      </c>
+      <c r="D103" s="2">
+        <v>60</v>
+      </c>
+      <c r="E103" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>46219</v>
+      </c>
+      <c r="B104" s="4">
+        <v>0.4375</v>
+      </c>
+      <c r="C104" t="s">
+        <v>1</v>
+      </c>
+      <c r="D104" s="2">
+        <v>60</v>
+      </c>
+      <c r="E104" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>46219</v>
+      </c>
+      <c r="B105" s="4">
+        <v>0.45</v>
+      </c>
+      <c r="C105" t="s">
+        <v>0</v>
+      </c>
+      <c r="D105" s="2">
+        <v>3634</v>
+      </c>
+      <c r="E105" t="s">
+        <v>22</v>
+      </c>
+      <c r="F105" s="2">
+        <v>83</v>
+      </c>
+      <c r="G105" s="2">
+        <v>784</v>
+      </c>
+      <c r="H105" s="3">
+        <v>6.01</v>
+      </c>
+      <c r="I105" s="2">
+        <v>7186</v>
+      </c>
+      <c r="J105" t="s">
+        <v>72</v>
+      </c>
+      <c r="K105" s="2">
+        <v>147</v>
+      </c>
+      <c r="L105" s="2">
+        <v>0</v>
+      </c>
+      <c r="M105" s="2">
+        <v>96</v>
+      </c>
+      <c r="N105" s="2">
+        <v>1</v>
+      </c>
+      <c r="O105" s="2">
+        <v>8</v>
+      </c>
+      <c r="P105" s="2">
+        <v>44</v>
+      </c>
+      <c r="Q105" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>46190</v>
+      </c>
+      <c r="B106" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C106" t="s">
+        <v>0</v>
+      </c>
+      <c r="D106" s="2">
+        <v>3687</v>
+      </c>
+      <c r="E106" t="s">
+        <v>22</v>
+      </c>
+      <c r="F106" s="2">
+        <v>51</v>
+      </c>
+      <c r="G106" s="2">
+        <v>672</v>
+      </c>
+      <c r="H106" s="3">
+        <v>5.37</v>
+      </c>
+      <c r="I106" s="2">
+        <v>6997</v>
+      </c>
+      <c r="J106" t="s">
+        <v>73</v>
+      </c>
+      <c r="K106" s="2">
+        <v>129</v>
+      </c>
+      <c r="L106" s="2">
+        <v>0</v>
+      </c>
+      <c r="M106" s="2">
+        <v>53</v>
+      </c>
+      <c r="N106" s="2">
+        <v>0</v>
+      </c>
+      <c r="O106" s="2">
+        <v>51</v>
+      </c>
+      <c r="P106" s="2">
+        <v>2</v>
+      </c>
+      <c r="Q106" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>46191</v>
+      </c>
+      <c r="B107" s="4">
+        <v>0.5625</v>
+      </c>
+      <c r="C107" t="s">
+        <v>2</v>
+      </c>
+      <c r="D107" s="2">
+        <v>60</v>
+      </c>
+      <c r="E107" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>46192</v>
+      </c>
+      <c r="B108" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="C108" t="s">
+        <v>1</v>
+      </c>
+      <c r="D108" s="2">
+        <v>60</v>
+      </c>
+      <c r="E108" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
2026-08-09 Hockey Predictions Fetch
</commit_message>
<xml_diff>
--- a/Python/Activities/data.xlsx
+++ b/Python/Activities/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Activities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24DCA9D0-19F1-4D56-9B93-8B080CCDC297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81DD15CE-EBC9-45A7-880F-5E95F2C6D458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{707279AB-A7E9-4A68-BEA1-90F4DD1BCF34}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="75">
   <si>
     <t>walk</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>11'26"</t>
+  </si>
+  <si>
+    <t>push-ups</t>
   </si>
 </sst>
 </file>
@@ -609,7 +612,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F196B904-6553-42BC-A222-B01279AC4ED1}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Q108"/>
+  <dimension ref="A1:Q125"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -4468,6 +4471,295 @@
         <v>3</v>
       </c>
     </row>
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>46228</v>
+      </c>
+      <c r="B109" s="4">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="C109" t="s">
+        <v>2</v>
+      </c>
+      <c r="D109" s="2">
+        <v>60</v>
+      </c>
+      <c r="E109" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>46233</v>
+      </c>
+      <c r="B110" s="4">
+        <v>0.6875</v>
+      </c>
+      <c r="C110" t="s">
+        <v>2</v>
+      </c>
+      <c r="D110" s="2">
+        <v>60</v>
+      </c>
+      <c r="E110" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>46235</v>
+      </c>
+      <c r="B111" s="4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C111" t="s">
+        <v>2</v>
+      </c>
+      <c r="D111" s="2">
+        <v>60</v>
+      </c>
+      <c r="E111" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>46236</v>
+      </c>
+      <c r="B112" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C112" t="s">
+        <v>2</v>
+      </c>
+      <c r="D112" s="2">
+        <v>60</v>
+      </c>
+      <c r="E112" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B113" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="C113" t="s">
+        <v>2</v>
+      </c>
+      <c r="D113" s="2">
+        <v>60</v>
+      </c>
+      <c r="E113" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>46238</v>
+      </c>
+      <c r="B114" s="4">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="C114" t="s">
+        <v>2</v>
+      </c>
+      <c r="D114" s="2">
+        <v>60</v>
+      </c>
+      <c r="E114" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>46239</v>
+      </c>
+      <c r="B115" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C115" t="s">
+        <v>74</v>
+      </c>
+      <c r="D115" s="2">
+        <v>25</v>
+      </c>
+      <c r="E115" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>46239</v>
+      </c>
+      <c r="B116" s="4">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C116" t="s">
+        <v>2</v>
+      </c>
+      <c r="D116" s="2">
+        <v>60</v>
+      </c>
+      <c r="E116" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>46240</v>
+      </c>
+      <c r="B117" s="4">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="C117" t="s">
+        <v>2</v>
+      </c>
+      <c r="D117" s="2">
+        <v>60</v>
+      </c>
+      <c r="E117" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>46240</v>
+      </c>
+      <c r="B118" s="4">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="C118" t="s">
+        <v>74</v>
+      </c>
+      <c r="D118" s="2">
+        <v>25</v>
+      </c>
+      <c r="E118" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>46241</v>
+      </c>
+      <c r="B119" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="C119" t="s">
+        <v>2</v>
+      </c>
+      <c r="D119" s="2">
+        <v>60</v>
+      </c>
+      <c r="E119" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>46242</v>
+      </c>
+      <c r="B120" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C120" t="s">
+        <v>74</v>
+      </c>
+      <c r="D120" s="2">
+        <v>25</v>
+      </c>
+      <c r="E120" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>46242</v>
+      </c>
+      <c r="B121" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C121" t="s">
+        <v>2</v>
+      </c>
+      <c r="D121" s="2">
+        <v>60</v>
+      </c>
+      <c r="E121" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>46242</v>
+      </c>
+      <c r="B122" s="4">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C122" t="s">
+        <v>1</v>
+      </c>
+      <c r="D122" s="2">
+        <v>60</v>
+      </c>
+      <c r="E122" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
+        <v>46243</v>
+      </c>
+      <c r="B123" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C123" t="s">
+        <v>74</v>
+      </c>
+      <c r="D123" s="2">
+        <v>25</v>
+      </c>
+      <c r="E123" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
+        <v>46243</v>
+      </c>
+      <c r="B124" s="4">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C124" t="s">
+        <v>2</v>
+      </c>
+      <c r="D124" s="2">
+        <v>60</v>
+      </c>
+      <c r="E124" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
+        <v>46243</v>
+      </c>
+      <c r="B125" s="4">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="C125" t="s">
+        <v>1</v>
+      </c>
+      <c r="D125" s="2">
+        <v>60</v>
+      </c>
+      <c r="E125" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q92" xr:uid="{F196B904-6553-42BC-A222-B01279AC4ED1}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>